<commit_message>
Address task 13.5-2 review feedback
</commit_message>
<xml_diff>
--- a/data/samples/platform_mappings.xlsx
+++ b/data/samples/platform_mappings.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" r:id="R1324e035280f4b23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="data" sheetId="1" r:id="Rb07027a2125f48d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -35,7 +35,7 @@
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="8">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -57,6 +57,21 @@
         <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="1">
     <x:border/>
@@ -64,7 +79,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="17">
+  <x:cellXfs count="33">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -101,6 +116,42 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -110,22 +161,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlatformMappings" displayName="PlatformMappings" ref="A1:N21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="14">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PlatformMappings" displayName="PlatformMappings" ref="A1:O21" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="15">
     <x:tableColumn id="1" name="mapping_id"/>
     <x:tableColumn id="2" name="mapping_kind"/>
     <x:tableColumn id="3" name="internal_sku"/>
-    <x:tableColumn id="4" name="platform_name"/>
-    <x:tableColumn id="5" name="platform_product_id"/>
-    <x:tableColumn id="6" name="platform_product_name"/>
-    <x:tableColumn id="7" name="normalized_platform_product_name"/>
-    <x:tableColumn id="8" name="grade"/>
-    <x:tableColumn id="9" name="search_keyword"/>
-    <x:tableColumn id="10" name="mapping_status"/>
-    <x:tableColumn id="11" name="effective_from"/>
-    <x:tableColumn id="12" name="effective_to"/>
-    <x:tableColumn id="13" name="last_verified_at"/>
-    <x:tableColumn id="14" name="remark"/>
+    <x:tableColumn id="4" name="candidate_internal_sku"/>
+    <x:tableColumn id="5" name="platform_name"/>
+    <x:tableColumn id="6" name="platform_product_id"/>
+    <x:tableColumn id="7" name="platform_product_name"/>
+    <x:tableColumn id="8" name="normalized_platform_product_name"/>
+    <x:tableColumn id="9" name="grade"/>
+    <x:tableColumn id="10" name="search_keyword"/>
+    <x:tableColumn id="11" name="mapping_status"/>
+    <x:tableColumn id="12" name="effective_from"/>
+    <x:tableColumn id="13" name="effective_to"/>
+    <x:tableColumn id="14" name="last_verified_at"/>
+    <x:tableColumn id="15" name="remark"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -329,723 +381,747 @@
     <x:col min="1" max="1" width="21" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="14" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="32" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="10" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="20" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="16" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="25" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="20" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="19" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="32" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="20" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="16" hidden="0" customWidth="1"/>
     <x:col min="12" max="12" width="22" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="22" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="44" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="22" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="48" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="34" customHeight="1">
-      <x:c r="A1" s="12" t="str">
+      <x:c r="A1" s="17" t="str">
         <x:v>mapping_id</x:v>
       </x:c>
-      <x:c r="B1" s="12" t="str">
+      <x:c r="B1" s="17" t="str">
         <x:v>mapping_kind</x:v>
       </x:c>
-      <x:c r="C1" s="12" t="str">
+      <x:c r="C1" s="17" t="str">
         <x:v>internal_sku</x:v>
       </x:c>
-      <x:c r="D1" s="12" t="str">
+      <x:c r="D1" s="17" t="str">
+        <x:v>candidate_internal_sku</x:v>
+      </x:c>
+      <x:c r="E1" s="17" t="str">
         <x:v>platform_name</x:v>
       </x:c>
-      <x:c r="E1" s="12" t="str">
+      <x:c r="F1" s="17" t="str">
         <x:v>platform_product_id</x:v>
       </x:c>
-      <x:c r="F1" s="12" t="str">
+      <x:c r="G1" s="17" t="str">
         <x:v>platform_product_name</x:v>
       </x:c>
-      <x:c r="G1" s="12" t="str">
+      <x:c r="H1" s="17" t="str">
         <x:v>normalized_platform_product_name</x:v>
       </x:c>
-      <x:c r="H1" s="12" t="str">
+      <x:c r="I1" s="17" t="str">
         <x:v>grade</x:v>
       </x:c>
-      <x:c r="I1" s="12" t="str">
+      <x:c r="J1" s="17" t="str">
         <x:v>search_keyword</x:v>
       </x:c>
-      <x:c r="J1" s="12" t="str">
+      <x:c r="K1" s="17" t="str">
         <x:v>mapping_status</x:v>
       </x:c>
-      <x:c r="K1" s="12" t="str">
+      <x:c r="L1" s="17" t="str">
         <x:v>effective_from</x:v>
       </x:c>
-      <x:c r="L1" s="12" t="str">
+      <x:c r="M1" s="17" t="str">
         <x:v>effective_to</x:v>
       </x:c>
-      <x:c r="M1" s="12" t="str">
+      <x:c r="N1" s="17" t="str">
         <x:v>last_verified_at</x:v>
       </x:c>
-      <x:c r="N1" s="12" t="str">
+      <x:c r="O1" s="17" t="str">
         <x:v>remark</x:v>
       </x:c>
     </x:row>
     <x:row r="2" ht="36" customHeight="1">
-      <x:c r="A2" s="13" t="str">
+      <x:c r="A2" s="23" t="str">
         <x:v>PLATFORM-01</x:v>
       </x:c>
-      <x:c r="B2" s="13" t="str">
+      <x:c r="B2" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C2" s="13" t="str"/>
-      <x:c r="D2" s="13" t="str">
+      <x:c r="C2" s="23"/>
+      <x:c r="D2" s="23" t="str"/>
+      <x:c r="E2" s="23" t="str">
         <x:v>寻梦</x:v>
       </x:c>
-      <x:c r="E2" s="13" t="str"/>
-      <x:c r="F2" s="13" t="str"/>
-      <x:c r="G2" s="13" t="str"/>
-      <x:c r="H2" s="13" t="str"/>
-      <x:c r="I2" s="13" t="str">
+      <x:c r="F2" s="23"/>
+      <x:c r="G2" s="23"/>
+      <x:c r="H2" s="23"/>
+      <x:c r="I2" s="23"/>
+      <x:c r="J2" s="23" t="str">
         <x:v>寻梦</x:v>
       </x:c>
-      <x:c r="J2" s="13" t="str">
+      <x:c r="K2" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K2" s="13" t="str"/>
-      <x:c r="L2" s="13" t="str"/>
-      <x:c r="M2" s="13" t="str"/>
-      <x:c r="N2" s="15" t="str">
+      <x:c r="L2" s="23"/>
+      <x:c r="M2" s="23"/>
+      <x:c r="N2" s="23"/>
+      <x:c r="O2" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" customHeight="1">
-      <x:c r="A3" s="13" t="str">
+      <x:c r="A3" s="23" t="str">
         <x:v>PLATFORM-02</x:v>
       </x:c>
-      <x:c r="B3" s="13" t="str">
+      <x:c r="B3" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C3" s="13" t="str"/>
-      <x:c r="D3" s="13" t="str">
+      <x:c r="C3" s="23"/>
+      <x:c r="D3" s="23" t="str"/>
+      <x:c r="E3" s="23" t="str">
         <x:v>花伍</x:v>
       </x:c>
-      <x:c r="E3" s="13" t="str"/>
-      <x:c r="F3" s="13" t="str"/>
-      <x:c r="G3" s="13" t="str"/>
-      <x:c r="H3" s="13" t="str"/>
-      <x:c r="I3" s="13" t="str">
+      <x:c r="F3" s="23"/>
+      <x:c r="G3" s="23"/>
+      <x:c r="H3" s="23"/>
+      <x:c r="I3" s="23"/>
+      <x:c r="J3" s="23" t="str">
         <x:v>花伍</x:v>
       </x:c>
-      <x:c r="J3" s="13" t="str">
+      <x:c r="K3" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K3" s="13" t="str"/>
-      <x:c r="L3" s="13" t="str"/>
-      <x:c r="M3" s="13" t="str"/>
-      <x:c r="N3" s="15" t="str">
+      <x:c r="L3" s="23"/>
+      <x:c r="M3" s="23"/>
+      <x:c r="N3" s="23"/>
+      <x:c r="O3" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="36" customHeight="1">
-      <x:c r="A4" s="13" t="str">
+      <x:c r="A4" s="23" t="str">
         <x:v>PLATFORM-03</x:v>
       </x:c>
-      <x:c r="B4" s="13" t="str">
+      <x:c r="B4" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C4" s="13" t="str"/>
-      <x:c r="D4" s="13" t="str">
+      <x:c r="C4" s="23"/>
+      <x:c r="D4" s="23" t="str"/>
+      <x:c r="E4" s="23" t="str">
         <x:v>珍情</x:v>
       </x:c>
-      <x:c r="E4" s="13" t="str"/>
-      <x:c r="F4" s="13" t="str"/>
-      <x:c r="G4" s="13" t="str"/>
-      <x:c r="H4" s="13" t="str"/>
-      <x:c r="I4" s="13" t="str">
+      <x:c r="F4" s="23"/>
+      <x:c r="G4" s="23"/>
+      <x:c r="H4" s="23"/>
+      <x:c r="I4" s="23"/>
+      <x:c r="J4" s="23" t="str">
         <x:v>珍情</x:v>
       </x:c>
-      <x:c r="J4" s="13" t="str">
+      <x:c r="K4" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K4" s="13" t="str"/>
-      <x:c r="L4" s="13" t="str"/>
-      <x:c r="M4" s="13" t="str"/>
-      <x:c r="N4" s="15" t="str">
+      <x:c r="L4" s="23"/>
+      <x:c r="M4" s="23"/>
+      <x:c r="N4" s="23"/>
+      <x:c r="O4" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" customHeight="1">
-      <x:c r="A5" s="13" t="str">
+      <x:c r="A5" s="23" t="str">
         <x:v>PLATFORM-04</x:v>
       </x:c>
-      <x:c r="B5" s="13" t="str">
+      <x:c r="B5" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C5" s="13" t="str"/>
-      <x:c r="D5" s="13" t="str">
+      <x:c r="C5" s="23"/>
+      <x:c r="D5" s="23" t="str"/>
+      <x:c r="E5" s="23" t="str">
         <x:v>花易宝</x:v>
       </x:c>
-      <x:c r="E5" s="13" t="str"/>
-      <x:c r="F5" s="13" t="str"/>
-      <x:c r="G5" s="13" t="str"/>
-      <x:c r="H5" s="13" t="str"/>
-      <x:c r="I5" s="13" t="str">
+      <x:c r="F5" s="23"/>
+      <x:c r="G5" s="23"/>
+      <x:c r="H5" s="23"/>
+      <x:c r="I5" s="23"/>
+      <x:c r="J5" s="23" t="str">
         <x:v>花易宝</x:v>
       </x:c>
-      <x:c r="J5" s="13" t="str">
+      <x:c r="K5" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K5" s="13" t="str"/>
-      <x:c r="L5" s="13" t="str"/>
-      <x:c r="M5" s="13" t="str"/>
-      <x:c r="N5" s="15" t="str">
+      <x:c r="L5" s="23"/>
+      <x:c r="M5" s="23"/>
+      <x:c r="N5" s="23"/>
+      <x:c r="O5" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="36" customHeight="1">
-      <x:c r="A6" s="13" t="str">
+      <x:c r="A6" s="23" t="str">
         <x:v>PLATFORM-05</x:v>
       </x:c>
-      <x:c r="B6" s="13" t="str">
+      <x:c r="B6" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C6" s="13" t="str"/>
-      <x:c r="D6" s="13" t="str">
+      <x:c r="C6" s="23"/>
+      <x:c r="D6" s="23" t="str"/>
+      <x:c r="E6" s="23" t="str">
         <x:v>蚂蚁</x:v>
       </x:c>
-      <x:c r="E6" s="13" t="str"/>
-      <x:c r="F6" s="13" t="str"/>
-      <x:c r="G6" s="13" t="str"/>
-      <x:c r="H6" s="13" t="str"/>
-      <x:c r="I6" s="13" t="str">
+      <x:c r="F6" s="23"/>
+      <x:c r="G6" s="23"/>
+      <x:c r="H6" s="23"/>
+      <x:c r="I6" s="23"/>
+      <x:c r="J6" s="23" t="str">
         <x:v>蚂蚁</x:v>
       </x:c>
-      <x:c r="J6" s="13" t="str">
+      <x:c r="K6" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K6" s="13" t="str"/>
-      <x:c r="L6" s="13" t="str"/>
-      <x:c r="M6" s="13" t="str"/>
-      <x:c r="N6" s="15" t="str">
+      <x:c r="L6" s="23"/>
+      <x:c r="M6" s="23"/>
+      <x:c r="N6" s="23"/>
+      <x:c r="O6" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="36" customHeight="1">
-      <x:c r="A7" s="13" t="str">
+      <x:c r="A7" s="23" t="str">
         <x:v>PLATFORM-06</x:v>
       </x:c>
-      <x:c r="B7" s="13" t="str">
+      <x:c r="B7" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C7" s="13" t="str"/>
-      <x:c r="D7" s="13" t="str">
+      <x:c r="C7" s="23"/>
+      <x:c r="D7" s="23" t="str"/>
+      <x:c r="E7" s="23" t="str">
         <x:v>花宝宝</x:v>
       </x:c>
-      <x:c r="E7" s="13" t="str"/>
-      <x:c r="F7" s="13" t="str"/>
-      <x:c r="G7" s="13" t="str"/>
-      <x:c r="H7" s="13" t="str"/>
-      <x:c r="I7" s="13" t="str">
+      <x:c r="F7" s="23"/>
+      <x:c r="G7" s="23"/>
+      <x:c r="H7" s="23"/>
+      <x:c r="I7" s="23"/>
+      <x:c r="J7" s="23" t="str">
         <x:v>花宝宝</x:v>
       </x:c>
-      <x:c r="J7" s="13" t="str">
+      <x:c r="K7" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K7" s="13" t="str"/>
-      <x:c r="L7" s="13" t="str"/>
-      <x:c r="M7" s="13" t="str"/>
-      <x:c r="N7" s="15" t="str">
+      <x:c r="L7" s="23"/>
+      <x:c r="M7" s="23"/>
+      <x:c r="N7" s="23"/>
+      <x:c r="O7" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="36" customHeight="1">
-      <x:c r="A8" s="13" t="str">
+      <x:c r="A8" s="23" t="str">
         <x:v>PLATFORM-07</x:v>
       </x:c>
-      <x:c r="B8" s="13" t="str">
+      <x:c r="B8" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C8" s="13" t="str"/>
-      <x:c r="D8" s="13" t="str">
+      <x:c r="C8" s="23"/>
+      <x:c r="D8" s="23" t="str"/>
+      <x:c r="E8" s="23" t="str">
         <x:v>花盛锦</x:v>
       </x:c>
-      <x:c r="E8" s="13" t="str"/>
-      <x:c r="F8" s="13" t="str"/>
-      <x:c r="G8" s="13" t="str"/>
-      <x:c r="H8" s="13" t="str"/>
-      <x:c r="I8" s="13" t="str">
+      <x:c r="F8" s="23"/>
+      <x:c r="G8" s="23"/>
+      <x:c r="H8" s="23"/>
+      <x:c r="I8" s="23"/>
+      <x:c r="J8" s="23" t="str">
         <x:v>花盛锦</x:v>
       </x:c>
-      <x:c r="J8" s="13" t="str">
+      <x:c r="K8" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K8" s="13" t="str"/>
-      <x:c r="L8" s="13" t="str"/>
-      <x:c r="M8" s="13" t="str"/>
-      <x:c r="N8" s="15" t="str">
+      <x:c r="L8" s="23"/>
+      <x:c r="M8" s="23"/>
+      <x:c r="N8" s="23"/>
+      <x:c r="O8" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="36" customHeight="1">
-      <x:c r="A9" s="13" t="str">
+      <x:c r="A9" s="23" t="str">
         <x:v>PLATFORM-08</x:v>
       </x:c>
-      <x:c r="B9" s="13" t="str">
+      <x:c r="B9" s="23" t="str">
         <x:v>PLATFORM</x:v>
       </x:c>
-      <x:c r="C9" s="13" t="str"/>
-      <x:c r="D9" s="13" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E9" s="13" t="str"/>
-      <x:c r="F9" s="13" t="str"/>
-      <x:c r="G9" s="13" t="str"/>
-      <x:c r="H9" s="13" t="str"/>
-      <x:c r="I9" s="13" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="J9" s="13" t="str">
+      <x:c r="C9" s="23"/>
+      <x:c r="D9" s="23" t="str"/>
+      <x:c r="E9" s="23" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F9" s="23"/>
+      <x:c r="G9" s="23"/>
+      <x:c r="H9" s="23"/>
+      <x:c r="I9" s="23"/>
+      <x:c r="J9" s="23" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="K9" s="23" t="str">
         <x:v>active</x:v>
       </x:c>
-      <x:c r="K9" s="13" t="str"/>
-      <x:c r="L9" s="13" t="str"/>
-      <x:c r="M9" s="13" t="str"/>
-      <x:c r="N9" s="15" t="str">
+      <x:c r="L9" s="23"/>
+      <x:c r="M9" s="23"/>
+      <x:c r="N9" s="23"/>
+      <x:c r="O9" s="24" t="str">
         <x:v>平台登记记录；供 WEB 运营表单选择，不参与商品身份解析。</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="36" customHeight="1">
-      <x:c r="A10" s="14" t="str">
+      <x:c r="A10" s="28" t="str">
         <x:v>MAYI-PRODUCT-01</x:v>
       </x:c>
-      <x:c r="B10" s="14" t="str">
+      <x:c r="B10" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C10" s="14" t="str">
+      <x:c r="C10" s="28" t="str"/>
+      <x:c r="D10" s="28" t="str">
         <x:v>AISHA-A-70-Z</x:v>
       </x:c>
-      <x:c r="D10" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E10" s="14" t="str"/>
-      <x:c r="F10" s="14" t="str">
+      <x:c r="E10" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F10" s="28"/>
+      <x:c r="G10" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="G10" s="14" t="str">
+      <x:c r="H10" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="H10" s="14" t="str">
+      <x:c r="I10" s="28" t="str">
         <x:v>A级</x:v>
       </x:c>
-      <x:c r="I10" s="14" t="str">
+      <x:c r="J10" s="28" t="str">
         <x:v>艾莎 A级</x:v>
       </x:c>
-      <x:c r="J10" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K10" s="14" t="str"/>
-      <x:c r="L10" s="14" t="str"/>
-      <x:c r="M10" s="14" t="str"/>
-      <x:c r="N10" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K10" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L10" s="28"/>
+      <x:c r="M10" s="28"/>
+      <x:c r="N10" s="28"/>
+      <x:c r="O10" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="36" customHeight="1">
-      <x:c r="A11" s="14" t="str">
+      <x:c r="A11" s="28" t="str">
         <x:v>MAYI-PRODUCT-02</x:v>
       </x:c>
-      <x:c r="B11" s="14" t="str">
+      <x:c r="B11" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C11" s="14" t="str">
+      <x:c r="C11" s="28" t="str"/>
+      <x:c r="D11" s="28" t="str">
         <x:v>AISHA-B-60-Z</x:v>
       </x:c>
-      <x:c r="D11" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E11" s="14" t="str"/>
-      <x:c r="F11" s="14" t="str">
+      <x:c r="E11" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F11" s="28"/>
+      <x:c r="G11" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="G11" s="14" t="str">
+      <x:c r="H11" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="H11" s="14" t="str">
+      <x:c r="I11" s="28" t="str">
         <x:v>B级</x:v>
       </x:c>
-      <x:c r="I11" s="14" t="str">
+      <x:c r="J11" s="28" t="str">
         <x:v>艾莎 B级</x:v>
       </x:c>
-      <x:c r="J11" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K11" s="14" t="str"/>
-      <x:c r="L11" s="14" t="str"/>
-      <x:c r="M11" s="14" t="str"/>
-      <x:c r="N11" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K11" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L11" s="28"/>
+      <x:c r="M11" s="28"/>
+      <x:c r="N11" s="28"/>
+      <x:c r="O11" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="36" customHeight="1">
-      <x:c r="A12" s="14" t="str">
+      <x:c r="A12" s="28" t="str">
         <x:v>MAYI-PRODUCT-03</x:v>
       </x:c>
-      <x:c r="B12" s="14" t="str">
+      <x:c r="B12" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C12" s="14" t="str">
+      <x:c r="C12" s="28" t="str"/>
+      <x:c r="D12" s="28" t="str">
         <x:v>AISHA-C-55-Z</x:v>
       </x:c>
-      <x:c r="D12" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E12" s="14" t="str"/>
-      <x:c r="F12" s="14" t="str">
+      <x:c r="E12" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F12" s="28"/>
+      <x:c r="G12" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="G12" s="14" t="str">
+      <x:c r="H12" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="H12" s="14" t="str">
+      <x:c r="I12" s="28" t="str">
         <x:v>C级</x:v>
       </x:c>
-      <x:c r="I12" s="14" t="str">
+      <x:c r="J12" s="28" t="str">
         <x:v>艾莎 C级</x:v>
       </x:c>
-      <x:c r="J12" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K12" s="14" t="str"/>
-      <x:c r="L12" s="14" t="str"/>
-      <x:c r="M12" s="14" t="str"/>
-      <x:c r="N12" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K12" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L12" s="28"/>
+      <x:c r="M12" s="28"/>
+      <x:c r="N12" s="28"/>
+      <x:c r="O12" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="36" customHeight="1">
-      <x:c r="A13" s="14" t="str">
+      <x:c r="A13" s="28" t="str">
         <x:v>MAYI-PRODUCT-04</x:v>
       </x:c>
-      <x:c r="B13" s="14" t="str">
+      <x:c r="B13" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C13" s="14" t="str">
+      <x:c r="C13" s="28" t="str"/>
+      <x:c r="D13" s="28" t="str">
         <x:v>AISHA-D-50-Z</x:v>
       </x:c>
-      <x:c r="D13" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E13" s="14" t="str"/>
-      <x:c r="F13" s="14" t="str">
+      <x:c r="E13" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F13" s="28"/>
+      <x:c r="G13" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="G13" s="14" t="str">
+      <x:c r="H13" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="H13" s="14" t="str">
+      <x:c r="I13" s="28" t="str">
         <x:v>D级</x:v>
       </x:c>
-      <x:c r="I13" s="14" t="str">
+      <x:c r="J13" s="28" t="str">
         <x:v>艾莎 D级</x:v>
       </x:c>
-      <x:c r="J13" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K13" s="14" t="str"/>
-      <x:c r="L13" s="14" t="str"/>
-      <x:c r="M13" s="14" t="str"/>
-      <x:c r="N13" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K13" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L13" s="28"/>
+      <x:c r="M13" s="28"/>
+      <x:c r="N13" s="28"/>
+      <x:c r="O13" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="36" customHeight="1">
-      <x:c r="A14" s="14" t="str">
+      <x:c r="A14" s="28" t="str">
         <x:v>MAYI-PRODUCT-05</x:v>
       </x:c>
-      <x:c r="B14" s="14" t="str">
+      <x:c r="B14" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C14" s="14" t="str">
+      <x:c r="C14" s="28" t="str"/>
+      <x:c r="D14" s="28" t="str">
         <x:v>AISHA-E-45-Z</x:v>
       </x:c>
-      <x:c r="D14" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E14" s="14" t="str"/>
-      <x:c r="F14" s="14" t="str">
+      <x:c r="E14" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F14" s="28"/>
+      <x:c r="G14" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="G14" s="14" t="str">
+      <x:c r="H14" s="28" t="str">
         <x:v>艾莎</x:v>
       </x:c>
-      <x:c r="H14" s="14" t="str">
+      <x:c r="I14" s="28" t="str">
         <x:v>E级</x:v>
       </x:c>
-      <x:c r="I14" s="14" t="str">
+      <x:c r="J14" s="28" t="str">
         <x:v>艾莎 E级</x:v>
       </x:c>
-      <x:c r="J14" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K14" s="14" t="str"/>
-      <x:c r="L14" s="14" t="str"/>
-      <x:c r="M14" s="14" t="str"/>
-      <x:c r="N14" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K14" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L14" s="28"/>
+      <x:c r="M14" s="28"/>
+      <x:c r="N14" s="28"/>
+      <x:c r="O14" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="36" customHeight="1">
-      <x:c r="A15" s="14" t="str">
+      <x:c r="A15" s="28" t="str">
         <x:v>MAYI-PRODUCT-06</x:v>
       </x:c>
-      <x:c r="B15" s="14" t="str">
+      <x:c r="B15" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C15" s="14" t="str">
+      <x:c r="C15" s="28" t="str"/>
+      <x:c r="D15" s="28" t="str">
         <x:v>CAPPUCCINO-A-70-Z</x:v>
       </x:c>
-      <x:c r="D15" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E15" s="14" t="str"/>
-      <x:c r="F15" s="14" t="str">
+      <x:c r="E15" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F15" s="28"/>
+      <x:c r="G15" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="G15" s="14" t="str">
+      <x:c r="H15" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="H15" s="14" t="str">
+      <x:c r="I15" s="28" t="str">
         <x:v>A级</x:v>
       </x:c>
-      <x:c r="I15" s="14" t="str">
+      <x:c r="J15" s="28" t="str">
         <x:v>卡布奇诺 A级</x:v>
       </x:c>
-      <x:c r="J15" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K15" s="14" t="str"/>
-      <x:c r="L15" s="14" t="str"/>
-      <x:c r="M15" s="14" t="str"/>
-      <x:c r="N15" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K15" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L15" s="28"/>
+      <x:c r="M15" s="28"/>
+      <x:c r="N15" s="28"/>
+      <x:c r="O15" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="36" customHeight="1">
-      <x:c r="A16" s="14" t="str">
+      <x:c r="A16" s="28" t="str">
         <x:v>MAYI-PRODUCT-07</x:v>
       </x:c>
-      <x:c r="B16" s="14" t="str">
+      <x:c r="B16" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C16" s="14" t="str">
+      <x:c r="C16" s="28" t="str"/>
+      <x:c r="D16" s="28" t="str">
         <x:v>CAPPUCCINO-B-60-Z</x:v>
       </x:c>
-      <x:c r="D16" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E16" s="14" t="str"/>
-      <x:c r="F16" s="14" t="str">
+      <x:c r="E16" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F16" s="28"/>
+      <x:c r="G16" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="G16" s="14" t="str">
+      <x:c r="H16" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="H16" s="14" t="str">
+      <x:c r="I16" s="28" t="str">
         <x:v>B级</x:v>
       </x:c>
-      <x:c r="I16" s="14" t="str">
+      <x:c r="J16" s="28" t="str">
         <x:v>卡布奇诺 B级</x:v>
       </x:c>
-      <x:c r="J16" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K16" s="14" t="str"/>
-      <x:c r="L16" s="14" t="str"/>
-      <x:c r="M16" s="14" t="str"/>
-      <x:c r="N16" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K16" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L16" s="28"/>
+      <x:c r="M16" s="28"/>
+      <x:c r="N16" s="28"/>
+      <x:c r="O16" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="36" customHeight="1">
-      <x:c r="A17" s="14" t="str">
+      <x:c r="A17" s="28" t="str">
         <x:v>MAYI-PRODUCT-08</x:v>
       </x:c>
-      <x:c r="B17" s="14" t="str">
+      <x:c r="B17" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C17" s="14" t="str">
+      <x:c r="C17" s="28" t="str"/>
+      <x:c r="D17" s="28" t="str">
         <x:v>CAPPUCCINO-C-55-Z</x:v>
       </x:c>
-      <x:c r="D17" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E17" s="14" t="str"/>
-      <x:c r="F17" s="14" t="str">
+      <x:c r="E17" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F17" s="28"/>
+      <x:c r="G17" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="G17" s="14" t="str">
+      <x:c r="H17" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="H17" s="14" t="str">
+      <x:c r="I17" s="28" t="str">
         <x:v>C级</x:v>
       </x:c>
-      <x:c r="I17" s="14" t="str">
+      <x:c r="J17" s="28" t="str">
         <x:v>卡布奇诺 C级</x:v>
       </x:c>
-      <x:c r="J17" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K17" s="14" t="str"/>
-      <x:c r="L17" s="14" t="str"/>
-      <x:c r="M17" s="14" t="str"/>
-      <x:c r="N17" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K17" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L17" s="28"/>
+      <x:c r="M17" s="28"/>
+      <x:c r="N17" s="28"/>
+      <x:c r="O17" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
-      <x:c r="A18" s="14" t="str">
+      <x:c r="A18" s="28" t="str">
         <x:v>MAYI-PRODUCT-09</x:v>
       </x:c>
-      <x:c r="B18" s="14" t="str">
+      <x:c r="B18" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C18" s="14" t="str">
+      <x:c r="C18" s="28" t="str"/>
+      <x:c r="D18" s="28" t="str">
         <x:v>CAPPUCCINO-D-50-Z</x:v>
       </x:c>
-      <x:c r="D18" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E18" s="14" t="str"/>
-      <x:c r="F18" s="14" t="str">
+      <x:c r="E18" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F18" s="28"/>
+      <x:c r="G18" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="G18" s="14" t="str">
+      <x:c r="H18" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="H18" s="14" t="str">
+      <x:c r="I18" s="28" t="str">
         <x:v>D级</x:v>
       </x:c>
-      <x:c r="I18" s="14" t="str">
+      <x:c r="J18" s="28" t="str">
         <x:v>卡布奇诺 D级</x:v>
       </x:c>
-      <x:c r="J18" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K18" s="14" t="str"/>
-      <x:c r="L18" s="14" t="str"/>
-      <x:c r="M18" s="14" t="str"/>
-      <x:c r="N18" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K18" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L18" s="28"/>
+      <x:c r="M18" s="28"/>
+      <x:c r="N18" s="28"/>
+      <x:c r="O18" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="36" customHeight="1">
-      <x:c r="A19" s="14" t="str">
+      <x:c r="A19" s="28" t="str">
         <x:v>MAYI-PRODUCT-10</x:v>
       </x:c>
-      <x:c r="B19" s="14" t="str">
+      <x:c r="B19" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C19" s="14" t="str">
+      <x:c r="C19" s="28" t="str"/>
+      <x:c r="D19" s="28" t="str">
         <x:v>CAPPUCCINO-E-45-Z</x:v>
       </x:c>
-      <x:c r="D19" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E19" s="14" t="str"/>
-      <x:c r="F19" s="14" t="str">
+      <x:c r="E19" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F19" s="28"/>
+      <x:c r="G19" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="G19" s="14" t="str">
+      <x:c r="H19" s="28" t="str">
         <x:v>卡布奇诺</x:v>
       </x:c>
-      <x:c r="H19" s="14" t="str">
+      <x:c r="I19" s="28" t="str">
         <x:v>E级</x:v>
       </x:c>
-      <x:c r="I19" s="14" t="str">
+      <x:c r="J19" s="28" t="str">
         <x:v>卡布奇诺 E级</x:v>
       </x:c>
-      <x:c r="J19" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K19" s="14" t="str"/>
-      <x:c r="L19" s="14" t="str"/>
-      <x:c r="M19" s="14" t="str"/>
-      <x:c r="N19" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K19" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L19" s="28"/>
+      <x:c r="M19" s="28"/>
+      <x:c r="N19" s="28"/>
+      <x:c r="O19" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="36" customHeight="1">
-      <x:c r="A20" s="14" t="str">
+      <x:c r="A20" s="28" t="str">
         <x:v>MAYI-PRODUCT-11</x:v>
       </x:c>
-      <x:c r="B20" s="14" t="str">
+      <x:c r="B20" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C20" s="14" t="str">
+      <x:c r="C20" s="28" t="str"/>
+      <x:c r="D20" s="28" t="str">
         <x:v>ZIXIA-0-FG-Z</x:v>
       </x:c>
-      <x:c r="D20" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E20" s="14" t="str"/>
-      <x:c r="F20" s="14" t="str">
+      <x:c r="E20" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F20" s="28"/>
+      <x:c r="G20" s="28" t="str">
         <x:v>紫霞仙子</x:v>
       </x:c>
-      <x:c r="G20" s="14" t="str">
+      <x:c r="H20" s="28" t="str">
         <x:v>紫霞仙子</x:v>
       </x:c>
-      <x:c r="H20" s="14" t="str">
+      <x:c r="I20" s="28" t="str">
         <x:v>0级</x:v>
       </x:c>
-      <x:c r="I20" s="14" t="str">
+      <x:c r="J20" s="28" t="str">
         <x:v>紫霞仙子 0级</x:v>
       </x:c>
-      <x:c r="J20" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K20" s="14" t="str"/>
-      <x:c r="L20" s="14" t="str"/>
-      <x:c r="M20" s="14" t="str"/>
-      <x:c r="N20" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K20" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L20" s="28"/>
+      <x:c r="M20" s="28"/>
+      <x:c r="N20" s="28"/>
+      <x:c r="O20" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="36" customHeight="1">
-      <x:c r="A21" s="14" t="str">
+      <x:c r="A21" s="28" t="str">
         <x:v>MAYI-PRODUCT-12</x:v>
       </x:c>
-      <x:c r="B21" s="14" t="str">
+      <x:c r="B21" s="28" t="str">
         <x:v>PRODUCT</x:v>
       </x:c>
-      <x:c r="C21" s="14" t="str">
+      <x:c r="C21" s="28" t="str"/>
+      <x:c r="D21" s="28" t="str">
         <x:v>ZIXIA-B-FG-Z</x:v>
       </x:c>
-      <x:c r="D21" s="14" t="str">
-        <x:v>蚂蚁花团供应商</x:v>
-      </x:c>
-      <x:c r="E21" s="14" t="str"/>
-      <x:c r="F21" s="14" t="str">
+      <x:c r="E21" s="28" t="str">
+        <x:v>蚂蚁花团供应商</x:v>
+      </x:c>
+      <x:c r="F21" s="28"/>
+      <x:c r="G21" s="28" t="str">
         <x:v>紫霞仙子</x:v>
       </x:c>
-      <x:c r="G21" s="14" t="str">
+      <x:c r="H21" s="28" t="str">
         <x:v>紫霞仙子</x:v>
       </x:c>
-      <x:c r="H21" s="14" t="str">
+      <x:c r="I21" s="28" t="str">
         <x:v>B级</x:v>
       </x:c>
-      <x:c r="I21" s="14" t="str">
+      <x:c r="J21" s="28" t="str">
         <x:v>紫霞仙子 B级</x:v>
       </x:c>
-      <x:c r="J21" s="14" t="str">
-        <x:v>VERIFIED</x:v>
-      </x:c>
-      <x:c r="K21" s="14" t="str"/>
-      <x:c r="L21" s="14" t="str"/>
-      <x:c r="M21" s="14" t="str"/>
-      <x:c r="N21" s="16" t="str">
-        <x:v>由 Task 13 只读扫描映射基线迁入；正式使用前仍需运营复核。</x:v>
+      <x:c r="K21" s="28" t="str">
+        <x:v>DISABLED</x:v>
+      </x:c>
+      <x:c r="L21" s="28"/>
+      <x:c r="M21" s="28"/>
+      <x:c r="N21" s="28"/>
+      <x:c r="O21" s="29" t="str">
+        <x:v>由 Task 13 只读扫描映射基线迁入；候选 SKU 待运营逐条复核后方可启用。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd026635cb54446c3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5b572e38f9e84408"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>